<commit_message>
Split weak and low pocket pair strategy rows
</commit_message>
<xml_diff>
--- a/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_strategy_8_categories.xlsx
+++ b/datasets/STU002__RNG001_UTG-vs-BB__BRD001_FLOP6/analysis/STU002_strategy_8_categories.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf8a169d0bd1d4243"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="Re0ff3912cd994ad1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="Rb8774f60859f4589"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="R151b5524444e4450"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R0b782f14a8c747bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="Re3295f6436824b90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="R80ce11b5dfac46ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="Rdd68c7f1ea7c4989"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2c67deb95bc74697"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 BB first" sheetId="2" r:id="R5ba1cab473a64c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 UTG cbet" sheetId="3" r:id="R50ba5b9af8374d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 BB vs cbet" sheetId="4" r:id="Rf3f16851f15141b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 UTG vs XR" sheetId="5" r:id="R1c44b24cac734ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 UTG vs donk" sheetId="6" r:id="R7fae541c6085498c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 BB vs donk R" sheetId="7" r:id="R4214f433b4e0403a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="8" r:id="Rc9f4db778b334c1d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -98,7 +98,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="11">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -133,6 +133,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F4F6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFEDD5"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -307,7 +312,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="91">
+  <x:cellXfs count="97">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -452,12 +457,27 @@
     <x:xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
@@ -485,46 +505,37 @@
     <x:xf numFmtId="0" fontId="11" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="8" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -539,19 +550,31 @@
     <x:xf numFmtId="0" fontId="11" fillId="10" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="10" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -817,7 +840,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="7" t="str">
-        <x:v>11 категорий рук × 8 категорий флопов. Чистое действие или строгий микс 50/50.</x:v>
+        <x:v>12 категорий рук × 8 категорий флопов. Чистое действие или строгий микс 50/50.</x:v>
       </x:c>
       <x:c r="B3" s="7"/>
       <x:c r="C3" s="7"/>
@@ -890,10 +913,10 @@
         <x:v>X 97.3%; D 2.7%</x:v>
       </x:c>
       <x:c r="F6" s="17" t="n">
-        <x:v>0.00020908534445406986</x:v>
+        <x:v>0.00020891461280731676</x:v>
       </x:c>
       <x:c r="G6" s="17" t="n">
-        <x:v>0.00020908534445406054</x:v>
+        <x:v>0.00020891461280730743</x:v>
       </x:c>
       <x:c r="H6" s="17" t="n">
         <x:v>-0.0000021173294650083556</x:v>
@@ -902,7 +925,7 @@
         <x:v>106381</x:v>
       </x:c>
       <x:c r="J6" s="18" t="n">
-        <x:v>77</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -919,22 +942,22 @@
         <x:v>X 44.1%; B 55.9%</x:v>
       </x:c>
       <x:c r="E7" s="15" t="str">
-        <x:v>X 38.2%; B 61.8%</x:v>
+        <x:v>X 39.3%; B 60.7%</x:v>
       </x:c>
       <x:c r="F7" s="17" t="n">
-        <x:v>0.0021102239420920476</x:v>
+        <x:v>0.0019001902633226213</x:v>
       </x:c>
       <x:c r="G7" s="17" t="n">
-        <x:v>0.0019756588678355256</x:v>
+        <x:v>0.0017790186479385063</x:v>
       </x:c>
       <x:c r="H7" s="17" t="n">
-        <x:v>0.00003344911351621407</x:v>
+        <x:v>0.00003381908454843101</x:v>
       </x:c>
       <x:c r="I7" s="18" t="n">
         <x:v>80553</x:v>
       </x:c>
       <x:c r="J7" s="18" t="n">
-        <x:v>81</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -951,22 +974,22 @@
         <x:v>F 47.9%; C 39.1%; R 13.0%</x:v>
       </x:c>
       <x:c r="E8" s="15" t="str">
-        <x:v>F 53.4%; C 36.9%; R 9.8%</x:v>
+        <x:v>F 52.5%; C 37.8%; R 9.8%</x:v>
       </x:c>
       <x:c r="F8" s="17" t="n">
-        <x:v>0.023656927129358886</x:v>
+        <x:v>0.02232512332335637</x:v>
       </x:c>
       <x:c r="G8" s="17" t="n">
-        <x:v>0.012382732642467134</x:v>
+        <x:v>0.0116856272926568</x:v>
       </x:c>
       <x:c r="H8" s="17" t="n">
-        <x:v>0.00229349091246097</x:v>
+        <x:v>0.0024426328877991243</x:v>
       </x:c>
       <x:c r="I8" s="18" t="n">
         <x:v>106308</x:v>
       </x:c>
       <x:c r="J8" s="18" t="n">
-        <x:v>77</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -983,22 +1006,22 @@
         <x:v>F 39.2%; C 60.8%</x:v>
       </x:c>
       <x:c r="E9" s="15" t="str">
-        <x:v>F 40.7%; C 59.3%</x:v>
+        <x:v>F 40.6%; C 59.4%</x:v>
       </x:c>
       <x:c r="F9" s="17" t="n">
-        <x:v>0.03569841486354705</x:v>
+        <x:v>0.034070487637216984</x:v>
       </x:c>
       <x:c r="G9" s="17" t="n">
-        <x:v>0.002430556988573247</x:v>
+        <x:v>0.0023197181764867862</x:v>
       </x:c>
       <x:c r="H9" s="17" t="n">
-        <x:v>0.00014985667236435806</x:v>
+        <x:v>0.00014957281499213037</x:v>
       </x:c>
       <x:c r="I9" s="18" t="n">
         <x:v>75236</x:v>
       </x:c>
       <x:c r="J9" s="18" t="n">
-        <x:v>81</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1018,19 +1041,19 @@
         <x:v>F 35.5%; C 58.5%; R 6.0%</x:v>
       </x:c>
       <x:c r="F10" s="17" t="n">
-        <x:v>0.016152337005416618</x:v>
+        <x:v>0.016253723985974047</x:v>
       </x:c>
       <x:c r="G10" s="17" t="n">
-        <x:v>0.001030004545578021</x:v>
+        <x:v>0.0010364698051130077</x:v>
       </x:c>
       <x:c r="H10" s="17" t="n">
-        <x:v>0.00001599728650821474</x:v>
+        <x:v>0.0000011934148435915806</x:v>
       </x:c>
       <x:c r="I10" s="18" t="n">
         <x:v>80553</x:v>
       </x:c>
       <x:c r="J10" s="18" t="n">
-        <x:v>81</x:v>
+        <x:v>88</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1047,22 +1070,22 @@
         <x:v>F 41.5%; C 58.5%</x:v>
       </x:c>
       <x:c r="E11" s="15" t="str">
-        <x:v>F 33.9%; C 66.1%</x:v>
+        <x:v>F 34.2%; C 65.8%</x:v>
       </x:c>
       <x:c r="F11" s="17" t="n">
-        <x:v>0.06378099211424014</x:v>
+        <x:v>0.054109096030611384</x:v>
       </x:c>
       <x:c r="G11" s="17" t="n">
-        <x:v>0.0005258479004592782</x:v>
+        <x:v>0.0004461071175011377</x:v>
       </x:c>
       <x:c r="H11" s="17" t="n">
-        <x:v>-0.000002422722774431422</x:v>
+        <x:v>-0.000002077152160189248</x:v>
       </x:c>
       <x:c r="I11" s="18" t="n">
         <x:v>57240</x:v>
       </x:c>
       <x:c r="J11" s="18" t="n">
-        <x:v>75</x:v>
+        <x:v>81</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1152,7 +1175,7 @@
       <x:c r="D16" s="23"/>
       <x:c r="E16" s="3"/>
       <x:c r="F16" s="24" t="str">
-        <x:v>11 категорий рук: 7 made, OESD, Gutshot, 2 overcards + BDFD и Air.</x:v>
+        <x:v>12 категорий рук: 8 made, OESD, Gutshot, 2 overcards + BDFD и Air.</x:v>
       </x:c>
       <x:c r="G16" s="24"/>
       <x:c r="H16" s="24"/>
@@ -1351,22 +1374,22 @@
       <x:c r="C5" s="31" t="str">
         <x:v>A-high medium (16)</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="59" t="str">
         <x:v>A-high low (28)</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="str">
+      <x:c r="E5" s="59" t="str">
         <x:v>Broadway (51)</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="str">
+      <x:c r="F5" s="59" t="str">
         <x:v>K/Q-high (56)</x:v>
       </x:c>
-      <x:c r="G5" s="54" t="str">
+      <x:c r="G5" s="59" t="str">
         <x:v>Middle dry (67)</x:v>
       </x:c>
-      <x:c r="H5" s="54" t="str">
+      <x:c r="H5" s="59" t="str">
         <x:v>Middle connected (26)</x:v>
       </x:c>
-      <x:c r="I5" s="54" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>Low (20)</x:v>
       </x:c>
     </x:row>
@@ -1378,22 +1401,22 @@
       <x:c r="C6" s="35" t="str">
         <x:v>A[J-T]x</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>A[9-2]x</x:v>
       </x:c>
-      <x:c r="E6" s="55" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>BBB BBx</x:v>
       </x:c>
-      <x:c r="F6" s="55" t="str">
+      <x:c r="F6" s="60" t="str">
         <x:v>K/Qx</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>[J-8]x dis</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="60" t="str">
         <x:v>[J-8]x con</x:v>
       </x:c>
-      <x:c r="I6" s="55" t="str">
+      <x:c r="I6" s="60" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
     </x:row>
@@ -1407,22 +1430,22 @@
       <x:c r="C7" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="D7" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E7" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F7" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G7" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H7" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I7" s="60" t="str">
+      <x:c r="D7" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E7" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F7" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G7" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H7" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I7" s="65" t="str">
         <x:v>D/X</x:v>
       </x:c>
     </x:row>
@@ -1436,22 +1459,22 @@
       <x:c r="C8" s="49" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G8" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H8" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I8" s="60" t="str">
+      <x:c r="D8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G8" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I8" s="65" t="str">
         <x:v>X/D</x:v>
       </x:c>
     </x:row>
@@ -1465,22 +1488,22 @@
       <x:c r="C9" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="D9" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E9" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F9" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G9" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H9" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I9" s="60" t="str">
+      <x:c r="D9" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F9" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H9" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I9" s="65" t="str">
         <x:v>X/D</x:v>
       </x:c>
     </x:row>
@@ -1494,22 +1517,22 @@
       <x:c r="C10" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="D10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I10" s="60" t="str">
+      <x:c r="D10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I10" s="65" t="str">
         <x:v>X/D</x:v>
       </x:c>
     </x:row>
@@ -1523,22 +1546,22 @@
       <x:c r="C11" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="D11" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E11" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F11" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G11" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H11" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I11" s="60" t="str">
+      <x:c r="D11" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E11" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F11" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G11" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H11" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I11" s="65" t="str">
         <x:v>X/D</x:v>
       </x:c>
     </x:row>
@@ -1552,167 +1575,196 @@
       <x:c r="C12" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="D12" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E12" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F12" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G12" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H12" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I12" s="60" t="str">
+      <x:c r="D12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I12" s="65" t="str">
         <x:v>X/D</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="C13" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="D13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I13" s="61" t="str">
+      <x:c r="B13" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C13" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H13" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I13" s="65" t="str">
+        <x:v>X/D</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Low pocket pair</x:v>
+      </x:c>
+      <x:c r="B14" s="55" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C14" s="55" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I14" s="66" t="str">
+        <x:v>D</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="37" t="str">
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B15" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C15" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D15" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F15" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G15" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H15" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I15" s="65" t="str">
         <x:v>D/X</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="37" t="str">
-        <x:v>OESD</x:v>
-      </x:c>
-      <x:c r="B14" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="C14" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="D14" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E14" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F14" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G14" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H14" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I14" s="60" t="str">
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="54" t="str">
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B16" s="55" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C16" s="55" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D16" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E16" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F16" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G16" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H16" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I16" s="67" t="str">
+        <x:v>X/D</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="54" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G17" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H17" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I17" s="67" t="str">
         <x:v>D/X</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="50" t="str">
-        <x:v>Gutshot</x:v>
-      </x:c>
-      <x:c r="B15" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="C15" s="51" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="D15" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E15" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F15" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G15" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H15" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I15" s="61" t="str">
-        <x:v>X/D</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="50" t="str">
-        <x:v>2 overcards + BDFD</x:v>
-      </x:c>
-      <x:c r="B16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H16" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I16" s="61" t="str">
-        <x:v>D/X</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="37" t="str">
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B17" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="C17" s="41" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="D17" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E17" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F17" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G17" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H17" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I17" s="56" t="str">
+      <x:c r="B18" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="C18" s="41" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="D18" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E18" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F18" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G18" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H18" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I18" s="61" t="str">
         <x:v>X</x:v>
       </x:c>
     </x:row>
@@ -1798,22 +1850,22 @@
       <x:c r="C5" s="31" t="str">
         <x:v>A-high medium (16)</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="59" t="str">
         <x:v>A-high low (28)</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="str">
+      <x:c r="E5" s="59" t="str">
         <x:v>Broadway (51)</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="str">
+      <x:c r="F5" s="59" t="str">
         <x:v>K/Q-high (56)</x:v>
       </x:c>
-      <x:c r="G5" s="54" t="str">
+      <x:c r="G5" s="59" t="str">
         <x:v>Middle dry (67)</x:v>
       </x:c>
-      <x:c r="H5" s="54" t="str">
+      <x:c r="H5" s="59" t="str">
         <x:v>Middle connected (26)</x:v>
       </x:c>
-      <x:c r="I5" s="54" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>Low (20)</x:v>
       </x:c>
     </x:row>
@@ -1825,22 +1877,22 @@
       <x:c r="C6" s="35" t="str">
         <x:v>A[J-T]x</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>A[9-2]x</x:v>
       </x:c>
-      <x:c r="E6" s="55" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>BBB BBx</x:v>
       </x:c>
-      <x:c r="F6" s="55" t="str">
+      <x:c r="F6" s="60" t="str">
         <x:v>K/Qx</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>[J-8]x dis</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="60" t="str">
         <x:v>[J-8]x con</x:v>
       </x:c>
-      <x:c r="I6" s="55" t="str">
+      <x:c r="I6" s="60" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
     </x:row>
@@ -1848,28 +1900,28 @@
       <x:c r="A7" s="37" t="str">
         <x:v>Two pair+</x:v>
       </x:c>
-      <x:c r="B7" s="65" t="str">
+      <x:c r="B7" s="71" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C7" s="65" t="str">
+      <x:c r="C7" s="71" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="D7" s="69" t="str">
+      <x:c r="D7" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="E7" s="69" t="str">
+      <x:c r="E7" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="F7" s="69" t="str">
+      <x:c r="F7" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G7" s="69" t="str">
+      <x:c r="G7" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="H7" s="69" t="str">
+      <x:c r="H7" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="I7" s="69" t="str">
+      <x:c r="I7" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -1883,22 +1935,22 @@
       <x:c r="C8" s="49" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E8" s="69" t="str">
+      <x:c r="D8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E8" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="F8" s="69" t="str">
+      <x:c r="F8" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G8" s="69" t="str">
+      <x:c r="G8" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="H8" s="69" t="str">
+      <x:c r="H8" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="I8" s="60" t="str">
+      <x:c r="I8" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
     </x:row>
@@ -1906,28 +1958,28 @@
       <x:c r="A9" s="37" t="str">
         <x:v>Top pair</x:v>
       </x:c>
-      <x:c r="B9" s="65" t="str">
+      <x:c r="B9" s="71" t="str">
         <x:v>B</x:v>
       </x:c>
       <x:c r="C9" s="45" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="D9" s="60" t="str">
+      <x:c r="D9" s="65" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="E9" s="69" t="str">
+      <x:c r="E9" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="F9" s="60" t="str">
+      <x:c r="F9" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="G9" s="60" t="str">
+      <x:c r="G9" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="H9" s="60" t="str">
+      <x:c r="H9" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="I9" s="69" t="str">
+      <x:c r="I9" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -1941,22 +1993,22 @@
       <x:c r="C10" s="41" t="str">
         <x:v>X</x:v>
       </x:c>
-      <x:c r="D10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="E10" s="60" t="str">
+      <x:c r="D10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E10" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="F10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G10" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H10" s="60" t="str">
+      <x:c r="F10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H10" s="65" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="I10" s="69" t="str">
+      <x:c r="I10" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -1970,22 +2022,22 @@
       <x:c r="C11" s="45" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="D11" s="69" t="str">
+      <x:c r="D11" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="E11" s="60" t="str">
+      <x:c r="E11" s="65" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="F11" s="69" t="str">
+      <x:c r="F11" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="G11" s="60" t="str">
+      <x:c r="G11" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="H11" s="60" t="str">
+      <x:c r="H11" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="I11" s="69" t="str">
+      <x:c r="I11" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
     </x:row>
@@ -1993,173 +2045,202 @@
       <x:c r="A12" s="37" t="str">
         <x:v>Third pair</x:v>
       </x:c>
-      <x:c r="B12" s="65" t="str">
+      <x:c r="B12" s="71" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C12" s="65" t="str">
+      <x:c r="C12" s="71" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="D12" s="69" t="str">
+      <x:c r="D12" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="E12" s="69" t="str">
+      <x:c r="E12" s="75" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="F12" s="60" t="str">
+      <x:c r="F12" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="G12" s="60" t="str">
+      <x:c r="G12" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="H12" s="56" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I12" s="60" t="str">
+      <x:c r="H12" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I12" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="66" t="str">
+      <x:c r="B13" s="45" t="str">
+        <x:v>B/X</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
+        <x:v>X/B</x:v>
+      </x:c>
+      <x:c r="D13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="E13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="F13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H13" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I13" s="61" t="str">
+        <x:v>X</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Low pocket pair</x:v>
+      </x:c>
+      <x:c r="B14" s="72" t="str">
         <x:v>B</x:v>
       </x:c>
-      <x:c r="C13" s="67" t="str">
+      <x:c r="C14" s="72" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D14" s="76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E14" s="76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="H14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I14" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="37" t="str">
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B15" s="71" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="C15" s="71" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D15" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E15" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F15" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G15" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H15" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I15" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="54" t="str">
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B16" s="72" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="C16" s="72" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="D16" s="76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="E16" s="76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F16" s="76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="G16" s="76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="H16" s="76" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="I16" s="67" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="D13" s="61" t="str">
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="54" t="str">
+        <x:v>2 overcards + BDFD</x:v>
+      </x:c>
+      <x:c r="B17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F17" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="G17" s="67" t="str">
+        <x:v>X/B</x:v>
+      </x:c>
+      <x:c r="H17" s="63" t="str">
+        <x:v>X</x:v>
+      </x:c>
+      <x:c r="I17" s="67" t="str">
+        <x:v>X/B</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="37" t="str">
+        <x:v>Air</x:v>
+      </x:c>
+      <x:c r="B18" s="45" t="str">
+        <x:v>X/B</x:v>
+      </x:c>
+      <x:c r="C18" s="45" t="str">
+        <x:v>X/B</x:v>
+      </x:c>
+      <x:c r="D18" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="E13" s="61" t="str">
+      <x:c r="E18" s="75" t="str">
+        <x:v>B</x:v>
+      </x:c>
+      <x:c r="F18" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-      <x:c r="F13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I13" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="37" t="str">
-        <x:v>OESD</x:v>
-      </x:c>
-      <x:c r="B14" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="C14" s="65" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="D14" s="69" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="E14" s="69" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="F14" s="69" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G14" s="69" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="H14" s="69" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="I14" s="69" t="str">
-        <x:v>B</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="50" t="str">
-        <x:v>Gutshot</x:v>
-      </x:c>
-      <x:c r="B15" s="66" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="C15" s="66" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="D15" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="E15" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="F15" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="G15" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="H15" s="70" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="I15" s="61" t="str">
+      <x:c r="G18" s="65" t="str">
         <x:v>B/X</x:v>
       </x:c>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="50" t="str">
-        <x:v>2 overcards + BDFD</x:v>
-      </x:c>
-      <x:c r="B16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G16" s="61" t="str">
+      <x:c r="H18" s="65" t="str">
         <x:v>X/B</x:v>
       </x:c>
-      <x:c r="H16" s="58" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I16" s="61" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="37" t="str">
-        <x:v>Air</x:v>
-      </x:c>
-      <x:c r="B17" s="45" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="C17" s="45" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="D17" s="60" t="str">
-        <x:v>B/X</x:v>
-      </x:c>
-      <x:c r="E17" s="69" t="str">
-        <x:v>B</x:v>
-      </x:c>
-      <x:c r="F17" s="60" t="str">
-        <x:v>B/X</x:v>
-      </x:c>
-      <x:c r="G17" s="60" t="str">
-        <x:v>B/X</x:v>
-      </x:c>
-      <x:c r="H17" s="60" t="str">
-        <x:v>X/B</x:v>
-      </x:c>
-      <x:c r="I17" s="60" t="str">
+      <x:c r="I18" s="65" t="str">
         <x:v>X/B</x:v>
       </x:c>
     </x:row>
@@ -2245,22 +2326,22 @@
       <x:c r="C5" s="31" t="str">
         <x:v>A-high medium (16)</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="59" t="str">
         <x:v>A-high low (28)</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="str">
+      <x:c r="E5" s="59" t="str">
         <x:v>Broadway (51)</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="str">
+      <x:c r="F5" s="59" t="str">
         <x:v>K/Q-high (56)</x:v>
       </x:c>
-      <x:c r="G5" s="54" t="str">
+      <x:c r="G5" s="59" t="str">
         <x:v>Middle dry (67)</x:v>
       </x:c>
-      <x:c r="H5" s="54" t="str">
+      <x:c r="H5" s="59" t="str">
         <x:v>Middle connected (26)</x:v>
       </x:c>
-      <x:c r="I5" s="54" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>Low (20)</x:v>
       </x:c>
     </x:row>
@@ -2272,22 +2353,22 @@
       <x:c r="C6" s="35" t="str">
         <x:v>A[J-T]x</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>A[9-2]x</x:v>
       </x:c>
-      <x:c r="E6" s="55" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>BBB BBx</x:v>
       </x:c>
-      <x:c r="F6" s="55" t="str">
+      <x:c r="F6" s="60" t="str">
         <x:v>K/Qx</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>[J-8]x dis</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="60" t="str">
         <x:v>[J-8]x con</x:v>
       </x:c>
-      <x:c r="I6" s="55" t="str">
+      <x:c r="I6" s="60" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
     </x:row>
@@ -2295,28 +2376,28 @@
       <x:c r="A7" s="37" t="str">
         <x:v>Two pair+</x:v>
       </x:c>
-      <x:c r="B7" s="74" t="str">
+      <x:c r="B7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="C7" s="74" t="str">
+      <x:c r="C7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="D7" s="80" t="str">
+      <x:c r="D7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="E7" s="80" t="str">
+      <x:c r="E7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="F7" s="80" t="str">
+      <x:c r="F7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="G7" s="80" t="str">
+      <x:c r="G7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="H7" s="80" t="str">
+      <x:c r="H7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="I7" s="80" t="str">
+      <x:c r="I7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
     </x:row>
@@ -2330,22 +2411,22 @@
       <x:c r="C8" s="49" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I8" s="56" t="str">
+      <x:c r="D8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I8" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2359,22 +2440,22 @@
       <x:c r="C9" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I9" s="56" t="str">
+      <x:c r="D9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I9" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2388,22 +2469,22 @@
       <x:c r="C10" s="45" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="D10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I10" s="56" t="str">
+      <x:c r="D10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I10" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2417,22 +2498,22 @@
       <x:c r="C11" s="45" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="D11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I11" s="56" t="str">
+      <x:c r="D11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I11" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2446,167 +2527,196 @@
       <x:c r="C12" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="D12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E12" s="60" t="str">
+      <x:c r="D12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E12" s="65" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="F12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I12" s="56" t="str">
+      <x:c r="F12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C13" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F13" s="81" t="str">
-        <x:v>F</x:v>
+      <x:c r="B13" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C13" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D13" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E13" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F13" s="65" t="str">
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="G13" s="61" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="H13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I13" s="58" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H13" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I13" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="37" t="str">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Low pocket pair</x:v>
+      </x:c>
+      <x:c r="B14" s="85" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C14" s="85" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I14" s="67" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="37" t="str">
         <x:v>OESD</x:v>
       </x:c>
-      <x:c r="B14" s="45" t="str">
+      <x:c r="B15" s="45" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="C14" s="74" t="str">
+      <x:c r="C15" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="D14" s="80" t="str">
+      <x:c r="D15" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="E14" s="60" t="str">
+      <x:c r="E15" s="65" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="F14" s="80" t="str">
+      <x:c r="F15" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="G14" s="80" t="str">
+      <x:c r="G15" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="H14" s="80" t="str">
+      <x:c r="H15" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="I14" s="80" t="str">
+      <x:c r="I15" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="50" t="str">
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="54" t="str">
         <x:v>Gutshot</x:v>
       </x:c>
-      <x:c r="B15" s="67" t="str">
+      <x:c r="B16" s="74" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="C15" s="67" t="str">
+      <x:c r="C16" s="74" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="D15" s="61" t="str">
+      <x:c r="D16" s="67" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="E15" s="61" t="str">
+      <x:c r="E16" s="67" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="F15" s="61" t="str">
+      <x:c r="F16" s="67" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="G15" s="61" t="str">
+      <x:c r="G16" s="67" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="H15" s="61" t="str">
+      <x:c r="H16" s="67" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="I15" s="61" t="str">
+      <x:c r="I16" s="67" t="str">
         <x:v>R/C</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="50" t="str">
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="54" t="str">
         <x:v>2 overcards + BDFD</x:v>
       </x:c>
-      <x:c r="B16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I16" s="61" t="str">
+      <x:c r="B17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I17" s="67" t="str">
         <x:v>C/F</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="37" t="str">
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B17" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C17" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I17" s="82" t="str">
+      <x:c r="B18" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C18" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I18" s="87" t="str">
         <x:v>F</x:v>
       </x:c>
     </x:row>
@@ -2692,22 +2802,22 @@
       <x:c r="C5" s="31" t="str">
         <x:v>A-high medium (16)</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="59" t="str">
         <x:v>A-high low (28)</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="str">
+      <x:c r="E5" s="59" t="str">
         <x:v>Broadway (51)</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="str">
+      <x:c r="F5" s="59" t="str">
         <x:v>K/Q-high (56)</x:v>
       </x:c>
-      <x:c r="G5" s="54" t="str">
+      <x:c r="G5" s="59" t="str">
         <x:v>Middle dry (67)</x:v>
       </x:c>
-      <x:c r="H5" s="54" t="str">
+      <x:c r="H5" s="59" t="str">
         <x:v>Middle connected (26)</x:v>
       </x:c>
-      <x:c r="I5" s="54" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>Low (20)</x:v>
       </x:c>
     </x:row>
@@ -2719,22 +2829,22 @@
       <x:c r="C6" s="35" t="str">
         <x:v>A[J-T]x</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>A[9-2]x</x:v>
       </x:c>
-      <x:c r="E6" s="55" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>BBB BBx</x:v>
       </x:c>
-      <x:c r="F6" s="55" t="str">
+      <x:c r="F6" s="60" t="str">
         <x:v>K/Qx</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>[J-8]x dis</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="60" t="str">
         <x:v>[J-8]x con</x:v>
       </x:c>
-      <x:c r="I6" s="55" t="str">
+      <x:c r="I6" s="60" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
     </x:row>
@@ -2748,22 +2858,22 @@
       <x:c r="C7" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I7" s="56" t="str">
+      <x:c r="D7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I7" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2777,22 +2887,22 @@
       <x:c r="C8" s="49" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I8" s="56" t="str">
+      <x:c r="D8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I8" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2806,22 +2916,22 @@
       <x:c r="C9" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I9" s="56" t="str">
+      <x:c r="D9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I9" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2835,22 +2945,22 @@
       <x:c r="C10" s="45" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="D10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I10" s="56" t="str">
+      <x:c r="D10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I10" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2858,28 +2968,28 @@
       <x:c r="A11" s="37" t="str">
         <x:v>Second pair</x:v>
       </x:c>
-      <x:c r="B11" s="78" t="str">
+      <x:c r="B11" s="84" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="C11" s="45" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="D11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I11" s="56" t="str">
+      <x:c r="D11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I11" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -2893,167 +3003,196 @@
       <x:c r="C12" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I12" s="56" t="str">
+      <x:c r="D12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C13" s="79" t="str">
+      <x:c r="B13" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C13" s="84" t="str">
         <x:v>F</x:v>
       </x:c>
       <x:c r="D13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E13" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H13" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Low pocket pair</x:v>
+      </x:c>
+      <x:c r="B14" s="85" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C14" s="85" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I14" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="37" t="str">
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B15" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C15" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="54" t="str">
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B16" s="55" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C16" s="74" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="E13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F13" s="61" t="str">
-        <x:v>F/C</x:v>
-      </x:c>
-      <x:c r="G13" s="61" t="str">
+      <x:c r="D16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E16" s="67" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="H13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I13" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="37" t="str">
-        <x:v>OESD</x:v>
-      </x:c>
-      <x:c r="B14" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C14" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="50" t="str">
-        <x:v>Gutshot</x:v>
-      </x:c>
-      <x:c r="B15" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C15" s="67" t="str">
-        <x:v>C/F</x:v>
-      </x:c>
-      <x:c r="D15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E15" s="61" t="str">
-        <x:v>C/F</x:v>
-      </x:c>
-      <x:c r="F15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="50" t="str">
+      <x:c r="F16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="54" t="str">
         <x:v>2 overcards + BDFD</x:v>
       </x:c>
-      <x:c r="B16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="37" t="str">
+      <x:c r="B17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B17" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C17" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I17" s="82" t="str">
+      <x:c r="B18" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C18" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I18" s="87" t="str">
         <x:v>F</x:v>
       </x:c>
     </x:row>
@@ -3139,22 +3278,22 @@
       <x:c r="C5" s="31" t="str">
         <x:v>A-high medium (16)</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="59" t="str">
         <x:v>A-high low (28)</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="str">
+      <x:c r="E5" s="59" t="str">
         <x:v>Broadway (51)</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="str">
+      <x:c r="F5" s="59" t="str">
         <x:v>K/Q-high (56)</x:v>
       </x:c>
-      <x:c r="G5" s="54" t="str">
+      <x:c r="G5" s="59" t="str">
         <x:v>Middle dry (67)</x:v>
       </x:c>
-      <x:c r="H5" s="54" t="str">
+      <x:c r="H5" s="59" t="str">
         <x:v>Middle connected (26)</x:v>
       </x:c>
-      <x:c r="I5" s="54" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>Low (20)</x:v>
       </x:c>
     </x:row>
@@ -3166,22 +3305,22 @@
       <x:c r="C6" s="35" t="str">
         <x:v>A[J-T]x</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>A[9-2]x</x:v>
       </x:c>
-      <x:c r="E6" s="55" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>BBB BBx</x:v>
       </x:c>
-      <x:c r="F6" s="55" t="str">
+      <x:c r="F6" s="60" t="str">
         <x:v>K/Qx</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>[J-8]x dis</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="60" t="str">
         <x:v>[J-8]x con</x:v>
       </x:c>
-      <x:c r="I6" s="55" t="str">
+      <x:c r="I6" s="60" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
     </x:row>
@@ -3189,28 +3328,28 @@
       <x:c r="A7" s="37" t="str">
         <x:v>Two pair+</x:v>
       </x:c>
-      <x:c r="B7" s="74" t="str">
+      <x:c r="B7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="C7" s="74" t="str">
+      <x:c r="C7" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="D7" s="60" t="str">
+      <x:c r="D7" s="65" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="E7" s="80" t="str">
+      <x:c r="E7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="F7" s="80" t="str">
+      <x:c r="F7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="G7" s="80" t="str">
+      <x:c r="G7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="H7" s="80" t="str">
+      <x:c r="H7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
-      <x:c r="I7" s="80" t="str">
+      <x:c r="I7" s="86" t="str">
         <x:v>R</x:v>
       </x:c>
     </x:row>
@@ -3224,22 +3363,22 @@
       <x:c r="C8" s="49" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E8" s="60" t="str">
+      <x:c r="D8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E8" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="F8" s="60" t="str">
+      <x:c r="F8" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="G8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I8" s="56" t="str">
+      <x:c r="G8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I8" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3253,22 +3392,22 @@
       <x:c r="C9" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I9" s="56" t="str">
+      <x:c r="D9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I9" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3282,22 +3421,22 @@
       <x:c r="C10" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E10" s="60" t="str">
+      <x:c r="D10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E10" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="F10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I10" s="56" t="str">
+      <x:c r="F10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I10" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3311,22 +3450,22 @@
       <x:c r="C11" s="45" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="D11" s="60" t="str">
+      <x:c r="D11" s="65" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="E11" s="60" t="str">
+      <x:c r="E11" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="F11" s="60" t="str">
+      <x:c r="F11" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="G11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I11" s="56" t="str">
+      <x:c r="G11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I11" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3334,173 +3473,202 @@
       <x:c r="A12" s="37" t="str">
         <x:v>Third pair</x:v>
       </x:c>
-      <x:c r="B12" s="74" t="str">
+      <x:c r="B12" s="80" t="str">
         <x:v>R</x:v>
       </x:c>
       <x:c r="C12" s="45" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="D12" s="60" t="str">
+      <x:c r="D12" s="65" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="E12" s="60" t="str">
+      <x:c r="E12" s="65" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="F12" s="60" t="str">
+      <x:c r="F12" s="65" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="G12" s="60" t="str">
+      <x:c r="G12" s="65" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="H12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I12" s="56" t="str">
+      <x:c r="H12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="67" t="str">
+      <x:c r="B13" s="45" t="str">
+        <x:v>F/R</x:v>
+      </x:c>
+      <x:c r="C13" s="45" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="C13" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E13" s="81" t="str">
-        <x:v>F</x:v>
+      <x:c r="D13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E13" s="65" t="str">
+        <x:v>C/F</x:v>
       </x:c>
       <x:c r="F13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H13" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="I13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Low pocket pair</x:v>
+      </x:c>
+      <x:c r="B14" s="85" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C14" s="85" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D14" s="67" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="E14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F14" s="67" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="G14" s="67" t="str">
+        <x:v>C/F</x:v>
+      </x:c>
+      <x:c r="H14" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I14" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="37" t="str">
+        <x:v>OESD</x:v>
+      </x:c>
+      <x:c r="B15" s="45" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="C15" s="45" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="D15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E15" s="65" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="F15" s="86" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="G15" s="86" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="H15" s="86" t="str">
+        <x:v>R</x:v>
+      </x:c>
+      <x:c r="I15" s="65" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="54" t="str">
+        <x:v>Gutshot</x:v>
+      </x:c>
+      <x:c r="B16" s="74" t="str">
+        <x:v>R/C</x:v>
+      </x:c>
+      <x:c r="C16" s="74" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="G13" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H13" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I13" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="37" t="str">
-        <x:v>OESD</x:v>
-      </x:c>
-      <x:c r="B14" s="45" t="str">
+      <x:c r="D16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E16" s="67" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="C14" s="45" t="str">
+      <x:c r="F16" s="67" t="str">
+        <x:v>C/R</x:v>
+      </x:c>
+      <x:c r="G16" s="67" t="str">
         <x:v>R/C</x:v>
       </x:c>
-      <x:c r="D14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E14" s="60" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="F14" s="80" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="G14" s="80" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="H14" s="80" t="str">
-        <x:v>R</x:v>
-      </x:c>
-      <x:c r="I14" s="60" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="50" t="str">
-        <x:v>Gutshot</x:v>
-      </x:c>
-      <x:c r="B15" s="67" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="C15" s="67" t="str">
+      <x:c r="H16" s="67" t="str">
         <x:v>C/R</x:v>
       </x:c>
-      <x:c r="D15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E15" s="61" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="F15" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="G15" s="61" t="str">
-        <x:v>R/C</x:v>
-      </x:c>
-      <x:c r="H15" s="61" t="str">
-        <x:v>C/R</x:v>
-      </x:c>
-      <x:c r="I15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="50" t="str">
+      <x:c r="I16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="54" t="str">
         <x:v>2 overcards + BDFD</x:v>
       </x:c>
-      <x:c r="B16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="37" t="str">
+      <x:c r="B17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B17" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C17" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F17" s="60" t="str">
+      <x:c r="B18" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C18" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F18" s="65" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="G17" s="60" t="str">
+      <x:c r="G18" s="65" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="H17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I17" s="82" t="str">
+      <x:c r="H18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I18" s="87" t="str">
         <x:v>F</x:v>
       </x:c>
     </x:row>
@@ -3586,22 +3754,22 @@
       <x:c r="C5" s="31" t="str">
         <x:v>A-high medium (16)</x:v>
       </x:c>
-      <x:c r="D5" s="54" t="str">
+      <x:c r="D5" s="59" t="str">
         <x:v>A-high low (28)</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="str">
+      <x:c r="E5" s="59" t="str">
         <x:v>Broadway (51)</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="str">
+      <x:c r="F5" s="59" t="str">
         <x:v>K/Q-high (56)</x:v>
       </x:c>
-      <x:c r="G5" s="54" t="str">
+      <x:c r="G5" s="59" t="str">
         <x:v>Middle dry (67)</x:v>
       </x:c>
-      <x:c r="H5" s="54" t="str">
+      <x:c r="H5" s="59" t="str">
         <x:v>Middle connected (26)</x:v>
       </x:c>
-      <x:c r="I5" s="54" t="str">
+      <x:c r="I5" s="59" t="str">
         <x:v>Low (20)</x:v>
       </x:c>
     </x:row>
@@ -3613,22 +3781,22 @@
       <x:c r="C6" s="35" t="str">
         <x:v>A[J-T]x</x:v>
       </x:c>
-      <x:c r="D6" s="55" t="str">
+      <x:c r="D6" s="60" t="str">
         <x:v>A[9-2]x</x:v>
       </x:c>
-      <x:c r="E6" s="55" t="str">
+      <x:c r="E6" s="60" t="str">
         <x:v>BBB BBx</x:v>
       </x:c>
-      <x:c r="F6" s="55" t="str">
+      <x:c r="F6" s="60" t="str">
         <x:v>K/Qx</x:v>
       </x:c>
-      <x:c r="G6" s="55" t="str">
+      <x:c r="G6" s="60" t="str">
         <x:v>[J-8]x dis</x:v>
       </x:c>
-      <x:c r="H6" s="55" t="str">
+      <x:c r="H6" s="60" t="str">
         <x:v>[J-8]x con</x:v>
       </x:c>
-      <x:c r="I6" s="55" t="str">
+      <x:c r="I6" s="60" t="str">
         <x:v>[7-4]x</x:v>
       </x:c>
     </x:row>
@@ -3642,22 +3810,22 @@
       <x:c r="C7" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H7" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I7" s="56" t="str">
+      <x:c r="D7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H7" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I7" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3671,22 +3839,22 @@
       <x:c r="C8" s="49" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="D8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F8" s="57" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H8" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I8" s="56" t="str">
+      <x:c r="D8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F8" s="62" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I8" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3700,22 +3868,22 @@
       <x:c r="C9" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="D9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H9" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I9" s="56" t="str">
+      <x:c r="D9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H9" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I9" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3726,25 +3894,25 @@
       <x:c r="B10" s="49" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="C10" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D10" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H10" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I10" s="56" t="str">
+      <x:c r="C10" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D10" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I10" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3755,25 +3923,25 @@
       <x:c r="B11" s="41" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="C11" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D11" s="60" t="str">
+      <x:c r="C11" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D11" s="65" t="str">
         <x:v>F/C</x:v>
       </x:c>
-      <x:c r="E11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H11" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I11" s="56" t="str">
+      <x:c r="E11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H11" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I11" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
@@ -3781,173 +3949,202 @@
       <x:c r="A12" s="37" t="str">
         <x:v>Third pair</x:v>
       </x:c>
-      <x:c r="B12" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C12" s="78" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D12" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E12" s="60" t="str">
+      <x:c r="B12" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C12" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D12" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E12" s="65" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="F12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H12" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I12" s="56" t="str">
+      <x:c r="F12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H12" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="str">
         <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="50" t="str">
+      <x:c r="A13" s="37" t="str">
         <x:v>Weak pair</x:v>
       </x:c>
-      <x:c r="B13" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="C13" s="79" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="D13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E13" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G13" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H13" s="81" t="str">
-        <x:v>F</x:v>
+      <x:c r="B13" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C13" s="84" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="D13" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E13" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F13" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G13" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H13" s="62" t="str">
+        <x:v>—</x:v>
       </x:c>
       <x:c r="I13" s="61" t="str">
-        <x:v>F/C</x:v>
+        <x:v>C</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="37" t="str">
+      <x:c r="A14" s="54" t="str">
+        <x:v>Low pocket pair</x:v>
+      </x:c>
+      <x:c r="B14" s="85" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="C14" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I14" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="37" t="str">
         <x:v>OESD</x:v>
       </x:c>
-      <x:c r="B14" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C14" s="41" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="F14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I14" s="56" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="50" t="str">
+      <x:c r="B15" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C15" s="41" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="F15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I15" s="61" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="54" t="str">
         <x:v>Gutshot</x:v>
       </x:c>
-      <x:c r="B15" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="C15" s="51" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="D15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="E15" s="61" t="str">
+      <x:c r="B16" s="55" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="C16" s="55" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="D16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="E16" s="67" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="F15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="G15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="I15" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="50" t="str">
+      <x:c r="F16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="G16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="I16" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="54" t="str">
         <x:v>2 overcards + BDFD</x:v>
       </x:c>
-      <x:c r="B16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C16" s="53" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="E16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="F16" s="59" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="G16" s="58" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="H16" s="61" t="str">
+      <x:c r="B17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="E17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="F17" s="64" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="G17" s="63" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="H17" s="67" t="str">
         <x:v>C/F</x:v>
       </x:c>
-      <x:c r="I16" s="81" t="str">
-        <x:v>F</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="37" t="str">
+      <x:c r="I17" s="88" t="str">
+        <x:v>F</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="37" t="str">
         <x:v>Air</x:v>
       </x:c>
-      <x:c r="B17" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="C17" s="49" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="D17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="E17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="F17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="G17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="H17" s="82" t="str">
-        <x:v>F</x:v>
-      </x:c>
-      <x:c r="I17" s="82" t="str">
+      <x:c r="B18" s="49" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="C18" s="49" t="str">
+        <x:v>—</x:v>
+      </x:c>
+      <x:c r="D18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="E18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="F18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="G18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="H18" s="87" t="str">
+        <x:v>F</x:v>
+      </x:c>
+      <x:c r="I18" s="87" t="str">
         <x:v>F</x:v>
       </x:c>
     </x:row>
@@ -3977,12 +4174,12 @@
       <x:c r="D1" s="3"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="84" t="str">
+      <x:c r="A2" s="90" t="str">
         <x:v>Методика</x:v>
       </x:c>
-      <x:c r="B2" s="84"/>
-      <x:c r="C2" s="84"/>
-      <x:c r="D2" s="84"/>
+      <x:c r="B2" s="90"/>
+      <x:c r="C2" s="90"/>
+      <x:c r="D2" s="90"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3"/>
@@ -4001,128 +4198,132 @@
       <x:c r="D4" s="21"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
-      <x:c r="A5" s="85" t="str">
+      <x:c r="A5" s="91" t="str">
         <x:v>Флопы</x:v>
       </x:c>
-      <x:c r="B5" s="85" t="str">
+      <x:c r="B5" s="91" t="str">
         <x:v>286 canonical unpaired rainbow flops, 8 итоговых категорий</x:v>
       </x:c>
       <x:c r="C5" s="3"/>
       <x:c r="D5" s="3"/>
     </x:row>
     <x:row r="6" ht="27" customHeight="1">
-      <x:c r="A6" s="85" t="str">
+      <x:c r="A6" s="91" t="str">
         <x:v>Диапазоны</x:v>
       </x:c>
-      <x:c r="B6" s="85" t="str">
+      <x:c r="B6" s="91" t="str">
         <x:v>RNG001: UTG open 2.5 bb / BB call из библиотеки TexasSolverGPU v0.2.0</x:v>
       </x:c>
       <x:c r="C6" s="3"/>
       <x:c r="D6" s="3"/>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
-      <x:c r="A7" s="85" t="str">
+      <x:c r="A7" s="91" t="str">
         <x:v>Частоты</x:v>
       </x:c>
-      <x:c r="B7" s="85" t="str">
+      <x:c r="B7" s="91" t="str">
         <x:v>Равное среднее по concrete combo на флопе, затем равное среднее по реальным флопам категории</x:v>
       </x:c>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
     </x:row>
     <x:row r="8" ht="27" customHeight="1">
-      <x:c r="A8" s="85" t="str">
+      <x:c r="A8" s="91" t="str">
         <x:v>Чистое действие</x:v>
       </x:c>
-      <x:c r="B8" s="85" t="str">
+      <x:c r="B8" s="91" t="str">
         <x:v>Наибольшая средняя частота строго &gt;65%</x:v>
       </x:c>
       <x:c r="C8" s="3"/>
       <x:c r="D8" s="3"/>
     </x:row>
     <x:row r="9" ht="27" customHeight="1">
-      <x:c r="A9" s="85" t="str">
+      <x:c r="A9" s="91" t="str">
         <x:v>Микс</x:v>
       </x:c>
-      <x:c r="B9" s="85" t="str">
+      <x:c r="B9" s="91" t="str">
         <x:v>Иначе два наиболее частых действия, строго 50/50; первым указано более частое действие солвера</x:v>
       </x:c>
       <x:c r="C9" s="3"/>
       <x:c r="D9" s="3"/>
     </x:row>
     <x:row r="10" ht="27" customHeight="1">
-      <x:c r="A10" s="85" t="str">
+      <x:c r="A10" s="91" t="str">
         <x:v>Вес диапазона</x:v>
       </x:c>
-      <x:c r="B10" s="85" t="str">
+      <x:c r="B10" s="91" t="str">
         <x:v>Combo с reach_probability &gt;0 участвует независимо от величины reach</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
-      <x:c r="A11" s="85" t="str">
+      <x:c r="A11" s="91" t="str">
         <x:v>EV-аудит</x:v>
       </x:c>
-      <x:c r="B11" s="85" t="str">
+      <x:c r="B11" s="91" t="str">
         <x:v>Reach-weighted local regret против solved opponent; не adaptive exploitability</x:v>
       </x:c>
       <x:c r="C11" s="3"/>
       <x:c r="D11" s="3"/>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
-      <x:c r="A12" s="85" t="str">
+      <x:c r="A12" s="91" t="str">
         <x:v>Категории рук</x:v>
       </x:c>
-      <x:c r="B12" s="85" t="str">
-        <x:v>7 made-категорий; затем OESD; Gutshot; 2 overcards + BDFD; Air</x:v>
+      <x:c r="B12" s="91" t="str">
+        <x:v>8 made-категорий; затем OESD; Gutshot; 2 overcards + BDFD; Air</x:v>
       </x:c>
       <x:c r="C12" s="3"/>
       <x:c r="D12" s="3"/>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
-      <x:c r="A13" s="85" t="str">
-        <x:v>Приоритет неготовых</x:v>
-      </x:c>
-      <x:c r="B13" s="85" t="str">
-        <x:v>OESD &gt; Gutshot &gt; 2 overcards + BDFD &gt; Air; BDFD без двух оверкарт уходит в Air</x:v>
+      <x:c r="A13" s="91" t="str">
+        <x:v>Карманные пары</x:v>
+      </x:c>
+      <x:c r="B13" s="91" t="str">
+        <x:v>Underpair: между top и middle; Weak pair: между middle и low; Low pocket pair: ниже low</x:v>
       </x:c>
       <x:c r="C13" s="3"/>
       <x:c r="D13" s="3"/>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
-      <x:c r="A14" s="85" t="str">
-        <x:v>Категории флопов</x:v>
-      </x:c>
-      <x:c r="B14" s="85" t="str">
-        <x:v>Восемь групп — итоговые категории; B13 только детерминированно задаёт их состав</x:v>
+      <x:c r="A14" s="91" t="str">
+        <x:v>Приоритет неготовых</x:v>
+      </x:c>
+      <x:c r="B14" s="91" t="str">
+        <x:v>OESD &gt; Gutshot &gt; 2 overcards + BDFD &gt; Air; BDFD без двух оверкарт уходит в Air</x:v>
       </x:c>
       <x:c r="C14" s="3"/>
       <x:c r="D14" s="3"/>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
-      <x:c r="A15" s="85" t="str">
-        <x:v>Роль исходной B13</x:v>
-      </x:c>
-      <x:c r="B15" s="85" t="str">
-        <x:v>Только детерминированное описание состава новых групп</x:v>
+      <x:c r="A15" s="91" t="str">
+        <x:v>Категории флопов</x:v>
+      </x:c>
+      <x:c r="B15" s="91" t="str">
+        <x:v>Восемь групп — итоговые категории; B13 только детерминированно задаёт их состав</x:v>
       </x:c>
       <x:c r="C15" s="3"/>
       <x:c r="D15" s="3"/>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
-      <x:c r="A16" s="85" t="str">
-        <x:v>JT9</x:v>
-      </x:c>
-      <x:c r="B16" s="85" t="str">
-        <x:v>Исходная B13 = [J-8]x con; в 8-групповой таблице = Middle connected</x:v>
+      <x:c r="A16" s="91" t="str">
+        <x:v>Роль исходной B13</x:v>
+      </x:c>
+      <x:c r="B16" s="91" t="str">
+        <x:v>Только детерминированное описание состава новых групп</x:v>
       </x:c>
       <x:c r="C16" s="3"/>
       <x:c r="D16" s="3"/>
     </x:row>
     <x:row r="17" ht="27" customHeight="1">
-      <x:c r="A17" s="3"/>
-      <x:c r="B17" s="3"/>
+      <x:c r="A17" s="91" t="str">
+        <x:v>JT9</x:v>
+      </x:c>
+      <x:c r="B17" s="91" t="str">
+        <x:v>Исходная B13 = [J-8]x con; в 8-групповой таблице = Middle connected</x:v>
+      </x:c>
       <x:c r="C17" s="3"/>
       <x:c r="D17" s="3"/>
     </x:row>
@@ -4133,136 +4334,136 @@
       <x:c r="D18" s="3"/>
     </x:row>
     <x:row r="19" ht="27" customHeight="1">
-      <x:c r="A19" s="86" t="str">
+      <x:c r="A19" s="3"/>
+      <x:c r="B19" s="3"/>
+      <x:c r="C19" s="3"/>
+      <x:c r="D19" s="3"/>
+    </x:row>
+    <x:row r="20" ht="27" customHeight="1">
+      <x:c r="A20" s="92" t="str">
         <x:v>Категория флопов</x:v>
       </x:c>
-      <x:c r="B19" s="86" t="str">
+      <x:c r="B20" s="92" t="str">
         <x:v>Входящие B13 / определение</x:v>
       </x:c>
-      <x:c r="C19" s="86" t="str">
+      <x:c r="C20" s="92" t="str">
         <x:v>Количество</x:v>
       </x:c>
-      <x:c r="D19" s="86" t="str">
+      <x:c r="D20" s="92" t="str">
         <x:v>Пояснение</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="27" customHeight="1">
-      <x:c r="A20" s="89" t="str">
+    <x:row r="21" ht="27" customHeight="1">
+      <x:c r="A21" s="95" t="str">
         <x:v>A-high high</x:v>
       </x:c>
-      <x:c r="B20" s="89" t="str">
+      <x:c r="B21" s="95" t="str">
         <x:v>ABB (6) + A[K/Q]x (16)</x:v>
       </x:c>
-      <x:c r="C20" s="90" t="n">
+      <x:c r="C21" s="96" t="n">
         <x:v>22</x:v>
       </x:c>
-      <x:c r="D20" s="89" t="str">
+      <x:c r="D21" s="95" t="str">
         <x:v>A с двумя broadway или с K/Q и младшей картой</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="27" customHeight="1">
-      <x:c r="A21" s="89" t="str">
+    <x:row r="22" ht="27" customHeight="1">
+      <x:c r="A22" s="95" t="str">
         <x:v>A-high medium</x:v>
       </x:c>
-      <x:c r="B21" s="89" t="str">
+      <x:c r="B22" s="95" t="str">
         <x:v>A[J-T][9-5] (10) + A[J-T][4-2] (6)</x:v>
       </x:c>
-      <x:c r="C21" s="90" t="n">
+      <x:c r="C22" s="96" t="n">
         <x:v>16</x:v>
       </x:c>
-      <x:c r="D21" s="89" t="str">
+      <x:c r="D22" s="95" t="str">
         <x:v>A с J/T</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="27" customHeight="1">
-      <x:c r="A22" s="89" t="str">
+    <x:row r="23" ht="27" customHeight="1">
+      <x:c r="A23" s="95" t="str">
         <x:v>A-high low</x:v>
       </x:c>
-      <x:c r="B22" s="89" t="str">
+      <x:c r="B23" s="95" t="str">
         <x:v>A[9-7]x (18) + A[6-2]x (10)</x:v>
       </x:c>
-      <x:c r="C22" s="90" t="n">
+      <x:c r="C23" s="96" t="n">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="D22" s="89" t="str">
+      <x:c r="D23" s="95" t="str">
         <x:v>A со средней картой 9 или ниже</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="27" customHeight="1">
-      <x:c r="A23" s="89" t="str">
+    <x:row r="24" ht="27" customHeight="1">
+      <x:c r="A24" s="95" t="str">
         <x:v>Broadway</x:v>
       </x:c>
-      <x:c r="B23" s="89" t="str">
+      <x:c r="B24" s="95" t="str">
         <x:v>BBB (4) + BBx (47)</x:v>
       </x:c>
-      <x:c r="C23" s="90" t="n">
+      <x:c r="C24" s="96" t="n">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="D23" s="89" t="str">
+      <x:c r="D24" s="95" t="str">
         <x:v>Без A; минимум две broadway-карты</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="27" customHeight="1">
-      <x:c r="A24" s="89" t="str">
+    <x:row r="25" ht="27" customHeight="1">
+      <x:c r="A25" s="95" t="str">
         <x:v>K/Q-high</x:v>
       </x:c>
-      <x:c r="B24" s="89" t="str">
+      <x:c r="B25" s="95" t="str">
         <x:v>K/Qx dis (42) + K/Qx con (14)</x:v>
       </x:c>
-      <x:c r="C24" s="90" t="n">
+      <x:c r="C25" s="96" t="n">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="D24" s="89" t="str">
+      <x:c r="D25" s="95" t="str">
         <x:v>Старшая K/Q, но не BBx</x:v>
       </x:c>
     </x:row>
-    <x:row r="25" ht="27" customHeight="1">
-      <x:c r="A25" s="89" t="str">
+    <x:row r="26" ht="27" customHeight="1">
+      <x:c r="A26" s="95" t="str">
         <x:v>Middle dry</x:v>
       </x:c>
-      <x:c r="B25" s="89" t="str">
+      <x:c r="B26" s="95" t="str">
         <x:v>[J-8]x dis (67)</x:v>
       </x:c>
-      <x:c r="C25" s="90" t="n">
+      <x:c r="C26" s="96" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="D25" s="89" t="str">
+      <x:c r="D26" s="95" t="str">
         <x:v>Старшая J/T/9/8; две младшие не соседние</x:v>
       </x:c>
     </x:row>
-    <x:row r="26" ht="27" customHeight="1">
-      <x:c r="A26" s="89" t="str">
+    <x:row r="27" ht="27" customHeight="1">
+      <x:c r="A27" s="95" t="str">
         <x:v>Middle connected</x:v>
       </x:c>
-      <x:c r="B26" s="89" t="str">
+      <x:c r="B27" s="95" t="str">
         <x:v>[J-8]x con (26)</x:v>
       </x:c>
-      <x:c r="C26" s="90" t="n">
+      <x:c r="C27" s="96" t="n">
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D26" s="89" t="str">
+      <x:c r="D27" s="95" t="str">
         <x:v>Старшая J/T/9/8; две младшие соседние; включает JT9</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="27" customHeight="1">
-      <x:c r="A27" s="89" t="str">
+    <x:row r="28" ht="27" customHeight="1">
+      <x:c r="A28" s="95" t="str">
         <x:v>Low</x:v>
       </x:c>
-      <x:c r="B27" s="89" t="str">
+      <x:c r="B28" s="95" t="str">
         <x:v>[7-4]x (20)</x:v>
       </x:c>
-      <x:c r="C27" s="90" t="n">
+      <x:c r="C28" s="96" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D27" s="89" t="str">
+      <x:c r="D28" s="95" t="str">
         <x:v>Старшая карта 7 или ниже</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28" ht="27" customHeight="1">
-      <x:c r="A28" s="3"/>
-      <x:c r="B28" s="3"/>
-      <x:c r="C28" s="3"/>
-      <x:c r="D28" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>